<commit_message>
-- AGREAGMOS MENU Y PAGINACION EJEMPLOS
</commit_message>
<xml_diff>
--- a/omitir/BD/EJEMPLOS.xlsx
+++ b/omitir/BD/EJEMPLOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\REPORTES_MENSUALES_2\omitir\BD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC296978-9DF1-4DFB-9712-8F8228A00139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF22C3CC-AA08-4EB0-8F79-BDF53C7348BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23040" yWindow="3300" windowWidth="20670" windowHeight="14295" xr2:uid="{11B3C740-C94D-4268-847C-642731C1E1BE}"/>
+    <workbookView xWindow="-23040" yWindow="1185" windowWidth="20670" windowHeight="14295" xr2:uid="{11B3C740-C94D-4268-847C-642731C1E1BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>ID</t>
   </si>
@@ -77,9 +77,6 @@
     <t>Comportamiento de la Red del Clie</t>
   </si>
   <si>
-    <t>INDICE CLIENTE</t>
-  </si>
-  <si>
     <t>ID CLIENTE</t>
   </si>
   <si>
@@ -90,14 +87,28 @@
   </si>
   <si>
     <t>GMG</t>
+  </si>
+  <si>
+    <t>Indice reportes</t>
+  </si>
+  <si>
+    <t>Pag reportes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -125,9 +136,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -464,13 +478,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{683F53B0-624C-4592-9FE8-9B4B9564B7D5}">
-  <dimension ref="B2:M25"/>
+  <dimension ref="B1:M25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="34.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="59" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+    </row>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
@@ -490,9 +514,11 @@
       <c r="G2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="L2" t="s">
-        <v>13</v>
-      </c>
+      <c r="J2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B3">
@@ -534,7 +560,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
@@ -560,10 +586,10 @@
         <v>73</v>
       </c>
       <c r="K5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L5" t="s">
         <v>15</v>
-      </c>
-      <c r="L5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
@@ -589,7 +615,7 @@
         <v>41</v>
       </c>
       <c r="K6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
@@ -933,6 +959,10 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="J2:L2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>